<commit_message>
Added more ddt tests and updated traker pages
</commit_message>
<xml_diff>
--- a/AMC_Master_Tracker.xlsx
+++ b/AMC_Master_Tracker.xlsx
@@ -9,6 +9,9 @@
     <sheet name="Priority Analysis" sheetId="4" r:id="rId4"/>
     <sheet name="Business Rules" sheetId="5" r:id="rId5"/>
     <sheet name="Data-Driven Results" sheetId="6" r:id="rId6"/>
+    <sheet name="DDT Attendance" sheetId="7" r:id="rId7"/>
+    <sheet name="DDT Leave Application" sheetId="8" r:id="rId8"/>
+    <sheet name="DDT Vendor" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -35325,7 +35328,7 @@
         <v>REJECTED</v>
       </c>
       <c r="D2" s="1" t="str">
-        <v>PAN must be unique</v>
+        <v>Your India Compliance API credits have exhaustedError fetching GSTIN details: Your India Compliance API credits have exhausted</v>
       </c>
       <c r="E2" s="1" t="str">
         <v>Review the highlighted field and correct the value</v>
@@ -35337,7 +35340,7 @@
         <v/>
       </c>
       <c r="H2" s="1" t="str">
-        <v>PAN must be unique</v>
+        <v>Your India Compliance API credits have exhaustedError fetching GSTIN details: Your India Compliance API credits have exhausted</v>
       </c>
     </row>
     <row r="3">
@@ -35403,7 +35406,7 @@
         <v>REJECTED</v>
       </c>
       <c r="D5" s="1" t="str">
-        <v>PAN must be unique</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure y</v>
       </c>
       <c r="E5" s="1" t="str">
         <v>Review the highlighted field and correct the value</v>
@@ -35415,7 +35418,7 @@
         <v/>
       </c>
       <c r="H5" s="1" t="str">
-        <v>PAN must be unique</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.</v>
       </c>
     </row>
     <row r="6">
@@ -35429,7 +35432,7 @@
         <v>REJECTED</v>
       </c>
       <c r="D6" s="1" t="str">
-        <v>GSTIN must be a valid 15-character GSTIN format (27ABC2DE1234F1Z5) or leave the field empty</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure y</v>
       </c>
       <c r="E6" s="1" t="str">
         <v>Review the highlighted field and correct the value</v>
@@ -35441,7 +35444,7 @@
         <v/>
       </c>
       <c r="H6" s="1" t="str">
-        <v>GSTIN must be a valid 15-character GSTIN format (27ABC2DE1234F1Z5) or leave the field empty</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.</v>
       </c>
     </row>
     <row r="7">
@@ -35478,7 +35481,7 @@
         <v>(empty)</v>
       </c>
       <c r="C8" s="1" t="str">
-        <v>SKIPPED</v>
+        <v>REJECTED</v>
       </c>
       <c r="D8" s="1" t="str">
         <v>Customer Name is required</v>
@@ -35490,10 +35493,10 @@
         <v>Customer Name is required</v>
       </c>
       <c r="G8" s="1" t="str">
-        <v>customer_name</v>
+        <v/>
       </c>
       <c r="H8" s="1" t="str">
-        <v>Customer Name is required</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.</v>
       </c>
     </row>
     <row r="9">
@@ -35533,7 +35536,7 @@
         <v>REJECTED</v>
       </c>
       <c r="D10" s="1" t="str">
-        <v>PAN must be unique</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure y</v>
       </c>
       <c r="E10" s="1" t="str">
         <v>Review the highlighted field and correct the value</v>
@@ -35545,7 +35548,7 @@
         <v/>
       </c>
       <c r="H10" s="1" t="str">
-        <v>PAN must be unique</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.</v>
       </c>
     </row>
     <row r="11">
@@ -35559,7 +35562,7 @@
         <v>REJECTED</v>
       </c>
       <c r="D11" s="1" t="str">
-        <v>PAN must be unique</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure y</v>
       </c>
       <c r="E11" s="1" t="str">
         <v>Review the highlighted field and correct the value</v>
@@ -35571,7 +35574,7 @@
         <v/>
       </c>
       <c r="H11" s="1" t="str">
-        <v>PAN must be unique</v>
+        <v>Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.Error fetching GSTIN details: Invalid GSTIN! The check digit validation has failed. Please ensure you've typed the GSTIN correctly.</v>
       </c>
     </row>
   </sheetData>
@@ -35579,4 +35582,661 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="str">
+        <v>Row</v>
+      </c>
+      <c r="B1" s="1" t="str">
+        <v>Key</v>
+      </c>
+      <c r="C1" s="1" t="str">
+        <v>Outcome</v>
+      </c>
+      <c r="D1" s="1" t="str">
+        <v>Reason</v>
+      </c>
+      <c r="E1" s="1" t="str">
+        <v>Pre-flight Issues</v>
+      </c>
+      <c r="F1" s="1" t="str">
+        <v>Raw Error</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="str">
+        <v>EMP-011</v>
+      </c>
+      <c r="C2" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D2" s="1" t="str">
+        <v>Beginning with Morning Shift You can use wildcard % txtNo ResultsCreate a new Shift Type More more</v>
+      </c>
+      <c r="E2" s="1" t="str">
+        <v>Unsupported status value: HOLIDAY</v>
+      </c>
+      <c r="F2" s="1" t="str">
+        <v>Beginning with Morning Shift You can use wildcard % txtNo ResultsCreate a new Shift Type More more</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>EMP-012</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <v>Mandatory fields required in AttendanceEmployeeCompany</v>
+      </c>
+      <c r="E3" s="1" t="str">
+        <v>Working Hours cannot be negative</v>
+      </c>
+      <c r="F3" s="1" t="str">
+        <v>Mandatory fields required in AttendanceEmployeeCompany</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>EMP-013</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>Mandatory fields required in AttendanceEmployeeCompany</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F4" s="1" t="str">
+        <v>Mandatory fields required in AttendanceEmployeeCompany</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>EMP-014</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <v>Mandatory fields required in AttendanceEmployeeCompany</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="1" t="str">
+        <v>Mandatory fields required in AttendanceEmployeeCompany</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="str">
+        <v>Row</v>
+      </c>
+      <c r="B1" s="1" t="str">
+        <v>Key</v>
+      </c>
+      <c r="C1" s="1" t="str">
+        <v>Outcome</v>
+      </c>
+      <c r="D1" s="1" t="str">
+        <v>Reason</v>
+      </c>
+      <c r="E1" s="1" t="str">
+        <v>Pre-flight Issues</v>
+      </c>
+      <c r="F1" s="1" t="str">
+        <v>Raw Error</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="str">
+        <v>EMP-005</v>
+      </c>
+      <c r="C2" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D2" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+      <c r="E2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F2" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>EMP-006</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+      <c r="E3" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F3" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>EMP-007</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F4" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>EMP-008</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="str">
+        <v>EMP-009</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+      <c r="E6" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <v>(empty employee)</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+      <c r="E7" s="1" t="str">
+        <v>Employee is required</v>
+      </c>
+      <c r="F7" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>11</v>
+      </c>
+      <c r="B8" s="1" t="str">
+        <v>EMP-011</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+      <c r="E8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>12</v>
+      </c>
+      <c r="B9" s="1" t="str">
+        <v>EMP-012</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+      <c r="E9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F9" s="1" t="str">
+        <v>Please select Employee first.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>13</v>
+      </c>
+      <c r="B10" s="1" t="str">
+        <v>EMP-013</v>
+      </c>
+      <c r="C10" s="1" t="str">
+        <v>ERROR</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <v>Save failed without visible ERPNext error</v>
+      </c>
+      <c r="E10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F10" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>14</v>
+      </c>
+      <c r="B11" s="1" t="str">
+        <v>EMP-014</v>
+      </c>
+      <c r="C11" s="1" t="str">
+        <v>ERROR</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <v>Save failed without visible ERPNext error</v>
+      </c>
+      <c r="E11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F11" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="str">
+        <v>Row</v>
+      </c>
+      <c r="B1" s="1" t="str">
+        <v>Key</v>
+      </c>
+      <c r="C1" s="1" t="str">
+        <v>Outcome</v>
+      </c>
+      <c r="D1" s="1" t="str">
+        <v>Reason</v>
+      </c>
+      <c r="E1" s="1" t="str">
+        <v>Pre-flight Issues</v>
+      </c>
+      <c r="F1" s="1" t="str">
+        <v>Raw Error</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="str">
+        <v>Apex HVAC Supplies Pvt Ltd</v>
+      </c>
+      <c r="C2" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D2" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F2" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>CoolTech Parts Private Limited</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E3" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F3" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>Suresh AC Services</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F4" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>Pinnacle Refrigeration Works</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="str">
+        <v>Delta Cooling Components</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E6" s="1" t="str">
+        <v>GST format is invalid</v>
+      </c>
+      <c r="F6" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <v>National Spares and Equipment</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E7" s="1" t="str">
+        <v>PAN format is invalid</v>
+      </c>
+      <c r="F7" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="str">
+        <v>Greenfield HVAC Solutions</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="str">
+        <v>Horizon Parts and Components</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D9" s="1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Message
+not-an-email is not a valid Email Address</v>
+      </c>
+      <c r="E9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F9" s="1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Message
+not-an-email is not a valid Email Address</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="str">
+        <v>Sunrise Equipment Suppliers</v>
+      </c>
+      <c r="C10" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="D10" s="1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Message
+98ABCD1234 is not a valid Phone Number</v>
+      </c>
+      <c r="E10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F10" s="1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Message
+98ABCD1234 is not a valid Phone Number</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="str">
+        <v>(empty supplier)</v>
+      </c>
+      <c r="C11" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E11" s="1" t="str">
+        <v>Supplier Name is required</v>
+      </c>
+      <c r="F11" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="str">
+        <v>Blue Star Vendor Network</v>
+      </c>
+      <c r="C12" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E12" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F12" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="str">
+        <v>Arctic HVAC Services Ltd</v>
+      </c>
+      <c r="C13" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E13" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F13" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="str">
+        <v>Polar Tech Maintenance</v>
+      </c>
+      <c r="C14" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D14" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E14" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F14" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="str">
+        <v>Summit HVAC Group India</v>
+      </c>
+      <c r="C15" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="D15" s="1" t="str">
+        <v>Vendor saved successfully</v>
+      </c>
+      <c r="E15" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F15" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added DDT scripts for service_calls and AMC contracts
</commit_message>
<xml_diff>
--- a/AMC_Master_Tracker.xlsx
+++ b/AMC_Master_Tracker.xlsx
@@ -12,6 +12,8 @@
     <sheet name="DDT Attendance" sheetId="7" r:id="rId7"/>
     <sheet name="DDT Leave Application" sheetId="8" r:id="rId8"/>
     <sheet name="DDT Vendor" sheetId="9" r:id="rId9"/>
+    <sheet name="DDT Service Call" sheetId="10" r:id="rId10"/>
+    <sheet name="DDT AMC Contract" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -7874,6 +7876,1094 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M13"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="str">
+        <v>Row</v>
+      </c>
+      <c r="B1" s="1" t="str">
+        <v>Test ID</v>
+      </c>
+      <c r="C1" s="1" t="str">
+        <v>Key</v>
+      </c>
+      <c r="D1" s="1" t="str">
+        <v>Expected Outcome</v>
+      </c>
+      <c r="E1" s="1" t="str">
+        <v>Actual Outcome</v>
+      </c>
+      <c r="F1" s="1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="G1" s="1" t="str">
+        <v>Reason</v>
+      </c>
+      <c r="H1" s="1" t="str">
+        <v>Selected Customer</v>
+      </c>
+      <c r="I1" s="1" t="str">
+        <v>Selected Branch</v>
+      </c>
+      <c r="J1" s="1" t="str">
+        <v>Selected Contact</v>
+      </c>
+      <c r="K1" s="1" t="str">
+        <v>Selected Type</v>
+      </c>
+      <c r="L1" s="1" t="str">
+        <v>Fallback Used</v>
+      </c>
+      <c r="M1" s="1" t="str">
+        <v>Raw Error</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="str">
+        <v>SC-DDT-001</v>
+      </c>
+      <c r="C2" s="1" t="str">
+        <v>Saffron Air Systems Pvt Ltd</v>
+      </c>
+      <c r="D2" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E2" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F2" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G2" s="1" t="str">
+        <v>Service Call saved successfully using available linked records (Using first complete customer hierarchy available in ERPNext)</v>
+      </c>
+      <c r="H2" s="1" t="str">
+        <v>Pricewaterhouse Coopers Private Limited</v>
+      </c>
+      <c r="I2" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J2" s="1" t="str">
+        <v>Shaikh yahya</v>
+      </c>
+      <c r="K2" s="1" t="str">
+        <v>Preventive maintenance</v>
+      </c>
+      <c r="L2" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M2" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>SC-DDT-002</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>Delta AMC Care</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E3" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F3" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G3" s="1" t="str">
+        <v>Service Call saved successfully using available linked records (Using first complete customer hierarchy available in ERPNext)</v>
+      </c>
+      <c r="H3" s="1" t="str">
+        <v>Pricewaterhouse Coopers Private Limited</v>
+      </c>
+      <c r="I3" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J3" s="1" t="str">
+        <v>Shaikh yahya</v>
+      </c>
+      <c r="K3" s="1" t="str">
+        <v>Breakdown</v>
+      </c>
+      <c r="L3" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M3" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>SC-DDT-003</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>Orbit Climate Works</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F4" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G4" s="1" t="str">
+        <v>Service Call saved successfully using available linked records</v>
+      </c>
+      <c r="H4" s="1" t="str">
+        <v>Pricewaterhouse Coopers Private Limited</v>
+      </c>
+      <c r="I4" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J4" s="1" t="str">
+        <v>Shaikh yahya</v>
+      </c>
+      <c r="K4" s="1" t="str">
+        <v>Installation</v>
+      </c>
+      <c r="L4" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M4" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>SC-DDT-004</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>Saffron Air Systems Pvt Ltd</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F5" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G5" s="1" t="str">
+        <v>Service Call saved successfully using available linked records (Using first complete customer hierarchy available in ERPNext)</v>
+      </c>
+      <c r="H5" s="1" t="str">
+        <v>Pricewaterhouse Coopers Private Limited</v>
+      </c>
+      <c r="I5" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J5" s="1" t="str">
+        <v>Shaikh yahya</v>
+      </c>
+      <c r="K5" s="1" t="str">
+        <v>Breakdown</v>
+      </c>
+      <c r="L5" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M5" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="str">
+        <v>SC-DDT-005</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <v>Delta AMC Care</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E6" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F6" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G6" s="1" t="str">
+        <v>Service Call saved successfully using available linked records (Using first complete customer hierarchy available in ERPNext)</v>
+      </c>
+      <c r="H6" s="1" t="str">
+        <v>Pricewaterhouse Coopers Private Limited</v>
+      </c>
+      <c r="I6" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J6" s="1" t="str">
+        <v>Shaikh yahya</v>
+      </c>
+      <c r="K6" s="1" t="str">
+        <v>Preventive maintenance</v>
+      </c>
+      <c r="L6" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M6" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <v>SC-DDT-006</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <v>Orbit Climate Works</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E7" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F7" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G7" s="1" t="str">
+        <v>Service Call saved successfully using available linked records</v>
+      </c>
+      <c r="H7" s="1" t="str">
+        <v>Pricewaterhouse Coopers Private Limited</v>
+      </c>
+      <c r="I7" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J7" s="1" t="str">
+        <v>Shaikh yahya</v>
+      </c>
+      <c r="K7" s="1" t="str">
+        <v>Breakdown</v>
+      </c>
+      <c r="L7" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M7" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="str">
+        <v>SC-DDT-007</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <v>Andheri Service Hub</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E8" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F8" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G8" s="1" t="str">
+        <v>Date Invalid date must be in format: dd-mm-yyyy</v>
+      </c>
+      <c r="H8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K8" s="1" t="str">
+        <v>Breakdown</v>
+      </c>
+      <c r="L8" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M8" s="1" t="str">
+        <v>Date Invalid date must be in format: dd-mm-yyyy</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="str">
+        <v>SC-DDT-008</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <v>Saffron Air Systems Pvt Ltd</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E9" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F9" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G9" s="1" t="str">
+        <v>Date Invalid date must be in format: dd-mm-yyyy</v>
+      </c>
+      <c r="H9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K9" s="1" t="str">
+        <v>Breakdown</v>
+      </c>
+      <c r="L9" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M9" s="1" t="str">
+        <v>Date Invalid date must be in format: dd-mm-yyyy</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="str">
+        <v>SC-DDT-009</v>
+      </c>
+      <c r="C10" s="1" t="str">
+        <v>Saffron Air Systems Pvt Ltd</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E10" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F10" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G10" s="1" t="str">
+        <v>Mandatory fields required in Service CallCustomerBranchContacted Person</v>
+      </c>
+      <c r="H10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K10" s="1" t="str">
+        <v>Breakdown</v>
+      </c>
+      <c r="L10" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M10" s="1" t="str">
+        <v>Mandatory fields required in Service CallCustomerBranchContacted Person</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="str">
+        <v>SC-DDT-010</v>
+      </c>
+      <c r="C11" s="1" t="str">
+        <v>Saffron Air Systems Pvt Ltd</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E11" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F11" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G11" s="1" t="str">
+        <v>Date Invalid date must be in format: dd-mm-yyyy</v>
+      </c>
+      <c r="H11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L11" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M11" s="1" t="str">
+        <v>Date Invalid date must be in format: dd-mm-yyyy</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="str">
+        <v>SC-DDT-011</v>
+      </c>
+      <c r="C12" s="1" t="str">
+        <v>Non Existing Customer</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E12" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F12" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G12" s="1" t="str">
+        <v>Date Invalid date must be in format: dd-mm-yyyy</v>
+      </c>
+      <c r="H12" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I12" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J12" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K12" s="1" t="str">
+        <v>Breakdown</v>
+      </c>
+      <c r="L12" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M12" s="1" t="str">
+        <v>Date Invalid date must be in format: dd-mm-yyyy</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="str">
+        <v>SC-DDT-012</v>
+      </c>
+      <c r="C13" s="1" t="str">
+        <v>Delta AMC Care</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E13" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F13" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G13" s="1" t="str">
+        <v>Service Call saved successfully using available linked records (Using first complete customer hierarchy available in ERPNext)</v>
+      </c>
+      <c r="H13" s="1" t="str">
+        <v>Pricewaterhouse Coopers Private Limited</v>
+      </c>
+      <c r="I13" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J13" s="1" t="str">
+        <v>Shaikh yahya</v>
+      </c>
+      <c r="K13" s="1" t="str">
+        <v>Installation</v>
+      </c>
+      <c r="L13" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M13" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M13"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="str">
+        <v>Row</v>
+      </c>
+      <c r="B1" s="1" t="str">
+        <v>Test ID</v>
+      </c>
+      <c r="C1" s="1" t="str">
+        <v>Key</v>
+      </c>
+      <c r="D1" s="1" t="str">
+        <v>Expected Outcome</v>
+      </c>
+      <c r="E1" s="1" t="str">
+        <v>Actual Outcome</v>
+      </c>
+      <c r="F1" s="1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="G1" s="1" t="str">
+        <v>Reason</v>
+      </c>
+      <c r="H1" s="1" t="str">
+        <v>Selected Customer</v>
+      </c>
+      <c r="I1" s="1" t="str">
+        <v>Selected Branch</v>
+      </c>
+      <c r="J1" s="1" t="str">
+        <v>Selected Contact</v>
+      </c>
+      <c r="K1" s="1" t="str">
+        <v>Applied Status</v>
+      </c>
+      <c r="L1" s="1" t="str">
+        <v>Fallback Used</v>
+      </c>
+      <c r="M1" s="1" t="str">
+        <v>Raw Error</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="str">
+        <v>CON-DDT-001</v>
+      </c>
+      <c r="C2" s="1" t="str">
+        <v>2030-04-01</v>
+      </c>
+      <c r="D2" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E2" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F2" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G2" s="1" t="str">
+        <v>AMC Contract saved successfully</v>
+      </c>
+      <c r="H2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K2" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L2" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M2" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>CON-DDT-002</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <v>2030-04-15</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E3" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F3" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G3" s="1" t="str">
+        <v>AMC Contract saved successfully</v>
+      </c>
+      <c r="H3" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I3" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J3" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K3" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L3" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M3" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="str">
+        <v>CON-DDT-003</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <v>2030-05-01</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E4" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F4" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G4" s="1" t="str">
+        <v>AMC Contract saved successfully</v>
+      </c>
+      <c r="H4" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I4" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J4" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K4" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L4" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M4" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v>CON-DDT-004</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <v>Saffron Air Systems Pvt Ltd</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F5" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G5" s="1" t="str">
+        <v>AMC Contract saved successfully with status Active using available linked records</v>
+      </c>
+      <c r="H5" s="1" t="str">
+        <v>Saffron Air Systems Pvt Ltd</v>
+      </c>
+      <c r="I5" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J5" s="1" t="str">
+        <v>Abdul Samad</v>
+      </c>
+      <c r="K5" s="1" t="str">
+        <v>Active</v>
+      </c>
+      <c r="L5" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M5" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="str">
+        <v>CON-DDT-005</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <v>Delta AMC Care</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E6" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F6" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G6" s="1" t="str">
+        <v>AMC Contract saved successfully with status Inactive using available linked records</v>
+      </c>
+      <c r="H6" s="1" t="str">
+        <v>Delta AMC Care</v>
+      </c>
+      <c r="I6" s="1" t="str">
+        <v>Cochin Branch</v>
+      </c>
+      <c r="J6" s="1" t="str">
+        <v>Abdul Samad</v>
+      </c>
+      <c r="K6" s="1" t="str">
+        <v>Inactive</v>
+      </c>
+      <c r="L6" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M6" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <v>CON-DDT-006</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <v>Orbit Climate Works</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="E7" s="1" t="str">
+        <v>CREATED</v>
+      </c>
+      <c r="F7" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G7" s="1" t="str">
+        <v>AMC Contract saved successfully using available linked records</v>
+      </c>
+      <c r="H7" s="1" t="str">
+        <v>Pricewaterhouse Coopers Private Limited</v>
+      </c>
+      <c r="I7" s="1" t="str">
+        <v>Mumbai Suburban</v>
+      </c>
+      <c r="J7" s="1" t="str">
+        <v>Abdul Samad</v>
+      </c>
+      <c r="K7" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L7" s="1" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M7" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="str">
+        <v>CON-DDT-007</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <v>(contract row)</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E8" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F8" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G8" s="1" t="str">
+        <v>Mandatory fields required in AMC ContractStart DateMandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2DateMandatory fields required in table Service Schedule, Row 3DateMandatory fields required in table Service Schedule, Row 4Date</v>
+      </c>
+      <c r="H8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K8" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L8" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M8" s="1" t="str">
+        <v>Mandatory fields required in AMC ContractStart DateMandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2DateMandatory fields required in table Service Schedule, Row 3DateMandatory fields required in table Service Schedule, Row 4Date</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="str">
+        <v>CON-DDT-008</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <v>2030-09-01</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E9" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F9" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G9" s="1" t="str">
+        <v>Mandatory fields required in AMC ContractEnd DateMandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2DateMandatory fields required in table Service Schedule, Row 3DateMandatory fields required in table Service Schedule, Row 4Date</v>
+      </c>
+      <c r="H9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K9" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L9" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M9" s="1" t="str">
+        <v>Mandatory fields required in AMC ContractEnd DateMandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2DateMandatory fields required in table Service Schedule, Row 3DateMandatory fields required in table Service Schedule, Row 4Date</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="str">
+        <v>CON-DDT-009</v>
+      </c>
+      <c r="C10" s="1" t="str">
+        <v>2030-10-01</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E10" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F10" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G10" s="1" t="str">
+        <v>Mandatory fields required in table Service Schedule, Row 1Date</v>
+      </c>
+      <c r="H10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K10" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L10" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M10" s="1" t="str">
+        <v>Mandatory fields required in table Service Schedule, Row 1Date</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="str">
+        <v>CON-DDT-010</v>
+      </c>
+      <c r="C11" s="1" t="str">
+        <v>2031-01-01</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E11" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F11" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G11" s="1" t="str">
+        <v>Mandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2DateMandatory fields required in table Service Schedule, Row 3DateMandatory fields required in table Service Schedule, Row 4Date</v>
+      </c>
+      <c r="H11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K11" s="1" t="str">
+        <v/>
+      </c>
+      <c r="L11" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M11" s="1" t="str">
+        <v>Mandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2DateMandatory fields required in table Service Schedule, Row 3DateMandatory fields required in table Service Schedule, Row 4Date</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="str">
+        <v>CON-DDT-011</v>
+      </c>
+      <c r="C12" s="1" t="str">
+        <v>Saffron Air Systems Pvt Ltd</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E12" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F12" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G12" s="1" t="str">
+        <v>Mandatory fields required in AMC ContractStart DateMandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2Date</v>
+      </c>
+      <c r="H12" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I12" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J12" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K12" s="1" t="str">
+        <v>Active</v>
+      </c>
+      <c r="L12" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M12" s="1" t="str">
+        <v>Mandatory fields required in AMC ContractStart DateMandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2Date</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="str">
+        <v>CON-DDT-012</v>
+      </c>
+      <c r="C13" s="1" t="str">
+        <v>Delta AMC Care</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="E13" s="1" t="str">
+        <v>REJECTED</v>
+      </c>
+      <c r="F13" s="1" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="G13" s="1" t="str">
+        <v>Mandatory fields required in AMC ContractEnd DateMandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2DateMandatory fields required in table Service Schedule, Row 3Date</v>
+      </c>
+      <c r="H13" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I13" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J13" s="1" t="str">
+        <v/>
+      </c>
+      <c r="K13" s="1" t="str">
+        <v>Inactive</v>
+      </c>
+      <c r="L13" s="1" t="str">
+        <v>No</v>
+      </c>
+      <c r="M13" s="1" t="str">
+        <v>Mandatory fields required in AMC ContractEnd DateMandatory fields required in table Service Schedule, Row 1DateMandatory fields required in table Service Schedule, Row 2DateMandatory fields required in table Service Schedule, Row 3Date</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O331"/>

</xml_diff>